<commit_message>
Update: implement Testcase_doc.xlsx for full version
</commit_message>
<xml_diff>
--- a/Testcase_doc.xlsx
+++ b/Testcase_doc.xlsx
@@ -19,7 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="93" uniqueCount="83">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="122" uniqueCount="91">
   <si>
     <t>Use case ID/ Req. ID</t>
   </si>
@@ -94,6 +94,27 @@
   </si>
   <si>
     <t>Defect Details</t>
+  </si>
+  <si>
+    <t>TC02</t>
+  </si>
+  <si>
+    <t>เมธอด return ผลลัพธ์เป็น &lt;valid&gt;</t>
+  </si>
+  <si>
+    <t>ปวริศช์ ประมวล</t>
+  </si>
+  <si>
+    <t>Open</t>
+  </si>
+  <si>
+    <t>High</t>
+  </si>
+  <si>
+    <t>TC03</t>
+  </si>
+  <si>
+    <t>TC04</t>
   </si>
   <si>
     <t>Test Scenario ID:</t>
@@ -181,7 +202,16 @@
     <t>1. message เป็นตัวอักษร A-Z จะให้ผลลัพธ์เป็น A-Z</t>
   </si>
   <si>
-    <t>เมธอด return ผลลัพธ์เป็น "VVIWZDUH"</t>
+    <t>เมธอด return ผลลัพธ์เป็น "VRIWZDUH"</t>
+  </si>
+  <si>
+    <t>VRIWZDUH</t>
+  </si>
+  <si>
+    <t>PASS</t>
+  </si>
+  <si>
+    <t>none</t>
   </si>
   <si>
     <t>2. message เป็นตัวอักษร a-z จะให้ผลลัพธ์เป็น a-z</t>
@@ -247,13 +277,10 @@
     <t>SOFTWARE</t>
   </si>
   <si>
-    <t>TC02</t>
-  </si>
-  <si>
     <t>software</t>
   </si>
   <si>
-    <t>TC03</t>
+    <t>invalid</t>
   </si>
   <si>
     <t>HELLO1</t>
@@ -262,19 +289,19 @@
     <t>เมธอด return ผลลัพธ์เป็น "KHOOR1"</t>
   </si>
   <si>
-    <t>TC04</t>
-  </si>
-  <si>
     <t>No1</t>
   </si>
   <si>
-    <t>เมธอด return ผลลัพธ์เป็น "Pq3"</t>
+    <t>เมธอด return ผลลัพธ์เป็น "QR1"</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <numFmts count="1">
+    <numFmt numFmtId="164" formatCode="m/d/yyyy"/>
+  </numFmts>
   <fonts count="9">
     <font>
       <sz val="11.0"/>
@@ -447,7 +474,7 @@
   <cellStyleXfs count="1">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
   </cellStyleXfs>
-  <cellXfs count="53">
+  <cellXfs count="55">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
@@ -482,8 +509,12 @@
     <xf borderId="1" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment readingOrder="0"/>
     </xf>
-    <xf borderId="1" fillId="4" fontId="1" numFmtId="0" xfId="0" applyBorder="1" applyFill="1" applyFont="1"/>
-    <xf borderId="1" fillId="5" fontId="1" numFmtId="0" xfId="0" applyBorder="1" applyFill="1" applyFont="1"/>
+    <xf borderId="1" fillId="4" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+      <alignment readingOrder="0"/>
+    </xf>
+    <xf borderId="1" fillId="5" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+      <alignment readingOrder="0"/>
+    </xf>
     <xf borderId="1" fillId="6" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment horizontal="center" shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
@@ -494,7 +525,10 @@
       <alignment horizontal="left" vertical="top"/>
     </xf>
     <xf borderId="1" fillId="0" fontId="6" numFmtId="14" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
-      <alignment horizontal="left" vertical="top"/>
+      <alignment horizontal="left" readingOrder="0" vertical="top"/>
+    </xf>
+    <xf borderId="1" fillId="0" fontId="6" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment horizontal="left" readingOrder="0" vertical="top"/>
     </xf>
     <xf borderId="1" fillId="0" fontId="7" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment shrinkToFit="0" vertical="center" wrapText="1"/>
@@ -511,8 +545,8 @@
     <xf borderId="5" fillId="0" fontId="7" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
-    <xf borderId="2" fillId="0" fontId="8" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment horizontal="center" shrinkToFit="0" vertical="center" wrapText="1"/>
+    <xf borderId="2" fillId="0" fontId="8" numFmtId="164" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
+      <alignment horizontal="center" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
     <xf borderId="2" fillId="7" fontId="7" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment horizontal="center"/>
@@ -538,8 +572,11 @@
     <xf borderId="5" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="left" readingOrder="0" vertical="top"/>
     </xf>
+    <xf borderId="1" fillId="0" fontId="8" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment readingOrder="0"/>
+    </xf>
+    <xf borderId="6" fillId="0" fontId="4" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
     <xf borderId="1" fillId="0" fontId="8" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
-    <xf borderId="6" fillId="0" fontId="4" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
     <xf borderId="7" fillId="0" fontId="4" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
     <xf borderId="1" fillId="0" fontId="7" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
     <xf borderId="2" fillId="0" fontId="8" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
@@ -906,10 +943,18 @@
       <c r="D3" s="7">
         <v>4.0</v>
       </c>
-      <c r="E3" s="5"/>
-      <c r="F3" s="5"/>
-      <c r="G3" s="5"/>
-      <c r="H3" s="5"/>
+      <c r="E3" s="7">
+        <v>1.0</v>
+      </c>
+      <c r="F3" s="7">
+        <v>3.0</v>
+      </c>
+      <c r="G3" s="7">
+        <v>0.0</v>
+      </c>
+      <c r="H3" s="7">
+        <v>0.0</v>
+      </c>
       <c r="I3" s="8" t="s">
         <v>10</v>
       </c>
@@ -1052,10 +1097,18 @@
       <c r="D8" s="13">
         <v>4.0</v>
       </c>
-      <c r="E8" s="14"/>
-      <c r="F8" s="15"/>
-      <c r="G8" s="9"/>
-      <c r="H8" s="9"/>
+      <c r="E8" s="14">
+        <v>1.0</v>
+      </c>
+      <c r="F8" s="15">
+        <v>3.0</v>
+      </c>
+      <c r="G8" s="13">
+        <v>0.0</v>
+      </c>
+      <c r="H8" s="13">
+        <v>0.0</v>
+      </c>
       <c r="I8" s="8" t="s">
         <v>13</v>
       </c>
@@ -28877,7 +28930,7 @@
   <cols>
     <col customWidth="1" min="1" max="1" width="9.29"/>
     <col customWidth="1" min="2" max="2" width="13.43"/>
-    <col customWidth="1" min="3" max="3" width="23.29"/>
+    <col customWidth="1" min="3" max="3" width="54.43"/>
     <col customWidth="1" min="4" max="4" width="14.43"/>
     <col customWidth="1" min="5" max="5" width="11.43"/>
     <col customWidth="1" min="6" max="6" width="16.71"/>
@@ -28928,16 +28981,88 @@
       <c r="A3" s="18">
         <v>1.0</v>
       </c>
-      <c r="B3" s="18"/>
-      <c r="C3" s="18"/>
-      <c r="D3" s="19"/>
+      <c r="B3" s="9" t="s">
+        <v>25</v>
+      </c>
+      <c r="C3" s="13" t="s">
+        <v>26</v>
+      </c>
+      <c r="D3" s="19">
+        <v>244568.0</v>
+      </c>
       <c r="E3" s="18"/>
-      <c r="F3" s="18"/>
-      <c r="G3" s="18"/>
-      <c r="H3" s="18"/>
-      <c r="I3" s="18"/>
+      <c r="F3" s="20" t="s">
+        <v>27</v>
+      </c>
+      <c r="G3" s="20" t="s">
+        <v>28</v>
+      </c>
+      <c r="H3" s="20" t="s">
+        <v>29</v>
+      </c>
+      <c r="I3" s="20" t="s">
+        <v>29</v>
+      </c>
       <c r="J3" s="18"/>
       <c r="K3" s="18"/>
+    </row>
+    <row r="4">
+      <c r="A4" s="20">
+        <v>2.0</v>
+      </c>
+      <c r="B4" s="13" t="s">
+        <v>30</v>
+      </c>
+      <c r="C4" s="13" t="s">
+        <v>26</v>
+      </c>
+      <c r="D4" s="19">
+        <v>244568.0</v>
+      </c>
+      <c r="E4" s="18"/>
+      <c r="F4" s="20" t="s">
+        <v>27</v>
+      </c>
+      <c r="G4" s="20" t="s">
+        <v>28</v>
+      </c>
+      <c r="H4" s="20" t="s">
+        <v>29</v>
+      </c>
+      <c r="I4" s="20" t="s">
+        <v>29</v>
+      </c>
+      <c r="J4" s="18"/>
+      <c r="K4" s="18"/>
+    </row>
+    <row r="5">
+      <c r="A5" s="20">
+        <v>3.0</v>
+      </c>
+      <c r="B5" s="13" t="s">
+        <v>31</v>
+      </c>
+      <c r="C5" s="13" t="s">
+        <v>26</v>
+      </c>
+      <c r="D5" s="19">
+        <v>244568.0</v>
+      </c>
+      <c r="E5" s="18"/>
+      <c r="F5" s="20" t="s">
+        <v>27</v>
+      </c>
+      <c r="G5" s="20" t="s">
+        <v>28</v>
+      </c>
+      <c r="H5" s="20" t="s">
+        <v>29</v>
+      </c>
+      <c r="I5" s="20" t="s">
+        <v>29</v>
+      </c>
+      <c r="J5" s="18"/>
+      <c r="K5" s="18"/>
     </row>
     <row r="21" ht="15.75" customHeight="1"/>
     <row r="22" ht="15.75" customHeight="1"/>
@@ -29946,86 +30071,88 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="20" t="s">
-        <v>25</v>
+      <c r="A1" s="21" t="s">
+        <v>32</v>
       </c>
-      <c r="B1" s="21" t="s">
-        <v>26</v>
+      <c r="B1" s="22" t="s">
+        <v>33</v>
       </c>
-      <c r="C1" s="20" t="s">
-        <v>27</v>
+      <c r="C1" s="21" t="s">
+        <v>34</v>
       </c>
-      <c r="D1" s="22" t="s">
-        <v>28</v>
+      <c r="D1" s="23" t="s">
+        <v>35</v>
       </c>
       <c r="E1" s="12"/>
     </row>
     <row r="2">
-      <c r="A2" s="20" t="s">
-        <v>29</v>
+      <c r="A2" s="21" t="s">
+        <v>36</v>
       </c>
-      <c r="B2" s="21" t="s">
+      <c r="B2" s="22" t="s">
         <v>11</v>
       </c>
-      <c r="C2" s="20" t="s">
-        <v>30</v>
+      <c r="C2" s="21" t="s">
+        <v>37</v>
       </c>
-      <c r="D2" s="22" t="s">
-        <v>31</v>
+      <c r="D2" s="23" t="s">
+        <v>38</v>
       </c>
       <c r="E2" s="12"/>
     </row>
     <row r="3">
-      <c r="A3" s="20" t="s">
-        <v>32</v>
+      <c r="A3" s="21" t="s">
+        <v>39</v>
       </c>
-      <c r="B3" s="21"/>
-      <c r="C3" s="20" t="s">
-        <v>33</v>
+      <c r="B3" s="22"/>
+      <c r="C3" s="21" t="s">
+        <v>40</v>
       </c>
-      <c r="D3" s="22" t="s">
-        <v>31</v>
+      <c r="D3" s="23" t="s">
+        <v>38</v>
       </c>
       <c r="E3" s="12"/>
     </row>
     <row r="4">
-      <c r="A4" s="20" t="s">
-        <v>34</v>
+      <c r="A4" s="21" t="s">
+        <v>41</v>
       </c>
-      <c r="B4" s="23" t="s">
-        <v>35</v>
+      <c r="B4" s="24" t="s">
+        <v>42</v>
       </c>
-      <c r="C4" s="24" t="s">
-        <v>36</v>
+      <c r="C4" s="25" t="s">
+        <v>43</v>
       </c>
-      <c r="D4" s="25"/>
+      <c r="D4" s="26">
+        <v>244568.0</v>
+      </c>
       <c r="E4" s="12"/>
     </row>
     <row r="5">
-      <c r="A5" s="20" t="s">
-        <v>37</v>
+      <c r="A5" s="21" t="s">
+        <v>44</v>
       </c>
-      <c r="B5" s="22" t="s">
-        <v>38</v>
+      <c r="B5" s="23" t="s">
+        <v>45</v>
       </c>
       <c r="C5" s="11"/>
       <c r="D5" s="11"/>
       <c r="E5" s="12"/>
     </row>
     <row r="6" ht="64.5" customHeight="1">
-      <c r="A6" s="24" t="s">
-        <v>39</v>
+      <c r="A6" s="25" t="s">
+        <v>46</v>
       </c>
-      <c r="B6" s="22" t="s">
-        <v>40</v>
+      <c r="B6" s="23" t="s">
+        <v>47</v>
       </c>
       <c r="C6" s="11"/>
       <c r="D6" s="11"/>
       <c r="E6" s="12"/>
     </row>
     <row r="7">
-      <c r="A7" s="26" t="s">
-        <v>41</v>
+      <c r="A7" s="27" t="s">
+        <v>48</v>
       </c>
       <c r="B7" s="11"/>
       <c r="C7" s="11"/>
@@ -30033,154 +30160,160 @@
       <c r="E7" s="12"/>
     </row>
     <row r="8">
-      <c r="A8" s="27" t="s">
-        <v>42</v>
+      <c r="A8" s="28" t="s">
+        <v>49</v>
       </c>
-      <c r="B8" s="27" t="s">
-        <v>43</v>
+      <c r="B8" s="28" t="s">
+        <v>50</v>
       </c>
-      <c r="C8" s="27" t="s">
-        <v>44</v>
+      <c r="C8" s="28" t="s">
+        <v>51</v>
       </c>
-      <c r="D8" s="27" t="s">
+      <c r="D8" s="28" t="s">
+        <v>52</v>
+      </c>
+      <c r="E8" s="28" t="s">
+        <v>53</v>
+      </c>
+      <c r="F8" s="29" t="s">
+        <v>54</v>
+      </c>
+      <c r="G8" s="29" t="s">
+        <v>55</v>
+      </c>
+      <c r="H8" s="29" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="9" ht="51.0" customHeight="1">
+      <c r="A9" s="30">
+        <v>1.0</v>
+      </c>
+      <c r="B9" s="31" t="s">
+        <v>57</v>
+      </c>
+      <c r="C9" s="32" t="s">
+        <v>58</v>
+      </c>
+      <c r="D9" s="33" t="s">
+        <v>59</v>
+      </c>
+      <c r="E9" s="34" t="s">
+        <v>60</v>
+      </c>
+      <c r="F9" s="13" t="s">
+        <v>61</v>
+      </c>
+      <c r="G9" s="35" t="s">
+        <v>62</v>
+      </c>
+      <c r="H9" s="35" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="36"/>
+      <c r="B10" s="36"/>
+      <c r="C10" s="37" t="s">
         <v>45</v>
       </c>
-      <c r="E8" s="27" t="s">
-        <v>46</v>
+      <c r="D10" s="33" t="s">
+        <v>64</v>
       </c>
-      <c r="F8" s="28" t="s">
-        <v>47</v>
+      <c r="E10" s="36"/>
+      <c r="F10" s="37"/>
+      <c r="G10" s="37"/>
+      <c r="H10" s="37"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="38"/>
+      <c r="B11" s="38"/>
+      <c r="C11" s="37"/>
+      <c r="D11" s="37" t="s">
+        <v>65</v>
       </c>
-      <c r="G8" s="28" t="s">
-        <v>48</v>
+      <c r="E11" s="38"/>
+      <c r="F11" s="37"/>
+      <c r="G11" s="37"/>
+      <c r="H11" s="37"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="37"/>
+      <c r="B12" s="37"/>
+      <c r="C12" s="37"/>
+      <c r="D12" s="37"/>
+      <c r="E12" s="37"/>
+      <c r="F12" s="37"/>
+      <c r="G12" s="37"/>
+      <c r="H12" s="37"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="37"/>
+      <c r="B13" s="37"/>
+      <c r="C13" s="37"/>
+      <c r="D13" s="37"/>
+      <c r="E13" s="37"/>
+      <c r="F13" s="37"/>
+      <c r="G13" s="37"/>
+      <c r="H13" s="37"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="37"/>
+      <c r="B14" s="37"/>
+      <c r="C14" s="37"/>
+      <c r="D14" s="37"/>
+      <c r="E14" s="37"/>
+      <c r="F14" s="37"/>
+      <c r="G14" s="37"/>
+      <c r="H14" s="37"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="37"/>
+      <c r="B15" s="37"/>
+      <c r="C15" s="37"/>
+      <c r="D15" s="37"/>
+      <c r="E15" s="37"/>
+      <c r="F15" s="37"/>
+      <c r="G15" s="37"/>
+      <c r="H15" s="37"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="37"/>
+      <c r="B16" s="37"/>
+      <c r="C16" s="37"/>
+      <c r="D16" s="37"/>
+      <c r="E16" s="37"/>
+      <c r="F16" s="37"/>
+      <c r="G16" s="37"/>
+      <c r="H16" s="37"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="37"/>
+      <c r="B17" s="37"/>
+      <c r="C17" s="37"/>
+      <c r="D17" s="37"/>
+      <c r="E17" s="37"/>
+      <c r="F17" s="37"/>
+      <c r="G17" s="37"/>
+      <c r="H17" s="37"/>
+    </row>
+    <row r="18">
+      <c r="A18" s="39" t="s">
+        <v>66</v>
       </c>
-      <c r="H8" s="28" t="s">
-        <v>49</v>
-      </c>
-    </row>
-    <row r="9" ht="51.0" customHeight="1">
-      <c r="A9" s="29">
-        <v>1.0</v>
-      </c>
-      <c r="B9" s="30" t="s">
-        <v>50</v>
-      </c>
-      <c r="C9" s="31" t="s">
-        <v>51</v>
-      </c>
-      <c r="D9" s="32" t="s">
-        <v>52</v>
-      </c>
-      <c r="E9" s="33" t="s">
-        <v>53</v>
-      </c>
-      <c r="F9" s="34"/>
-      <c r="G9" s="34"/>
-      <c r="H9" s="34"/>
-    </row>
-    <row r="10">
-      <c r="A10" s="35"/>
-      <c r="B10" s="35"/>
-      <c r="C10" s="34" t="s">
-        <v>38</v>
-      </c>
-      <c r="D10" s="32" t="s">
-        <v>54</v>
-      </c>
-      <c r="E10" s="35"/>
-      <c r="F10" s="34"/>
-      <c r="G10" s="34"/>
-      <c r="H10" s="34"/>
-    </row>
-    <row r="11">
-      <c r="A11" s="36"/>
-      <c r="B11" s="36"/>
-      <c r="C11" s="34"/>
-      <c r="D11" s="34" t="s">
-        <v>55</v>
-      </c>
-      <c r="E11" s="36"/>
-      <c r="F11" s="34"/>
-      <c r="G11" s="34"/>
-      <c r="H11" s="34"/>
-    </row>
-    <row r="12">
-      <c r="A12" s="34"/>
-      <c r="B12" s="34"/>
-      <c r="C12" s="34"/>
-      <c r="D12" s="34"/>
-      <c r="E12" s="34"/>
-      <c r="F12" s="34"/>
-      <c r="G12" s="34"/>
-      <c r="H12" s="34"/>
-    </row>
-    <row r="13">
-      <c r="A13" s="34"/>
-      <c r="B13" s="34"/>
-      <c r="C13" s="34"/>
-      <c r="D13" s="34"/>
-      <c r="E13" s="34"/>
-      <c r="F13" s="34"/>
-      <c r="G13" s="34"/>
-      <c r="H13" s="34"/>
-    </row>
-    <row r="14">
-      <c r="A14" s="34"/>
-      <c r="B14" s="34"/>
-      <c r="C14" s="34"/>
-      <c r="D14" s="34"/>
-      <c r="E14" s="34"/>
-      <c r="F14" s="34"/>
-      <c r="G14" s="34"/>
-      <c r="H14" s="34"/>
-    </row>
-    <row r="15">
-      <c r="A15" s="34"/>
-      <c r="B15" s="34"/>
-      <c r="C15" s="34"/>
-      <c r="D15" s="34"/>
-      <c r="E15" s="34"/>
-      <c r="F15" s="34"/>
-      <c r="G15" s="34"/>
-      <c r="H15" s="34"/>
-    </row>
-    <row r="16">
-      <c r="A16" s="34"/>
-      <c r="B16" s="34"/>
-      <c r="C16" s="34"/>
-      <c r="D16" s="34"/>
-      <c r="E16" s="34"/>
-      <c r="F16" s="34"/>
-      <c r="G16" s="34"/>
-      <c r="H16" s="34"/>
-    </row>
-    <row r="17">
-      <c r="A17" s="34"/>
-      <c r="B17" s="34"/>
-      <c r="C17" s="34"/>
-      <c r="D17" s="34"/>
-      <c r="E17" s="34"/>
-      <c r="F17" s="34"/>
-      <c r="G17" s="34"/>
-      <c r="H17" s="34"/>
-    </row>
-    <row r="18">
-      <c r="A18" s="37" t="s">
-        <v>56</v>
-      </c>
-      <c r="B18" s="38" t="s">
-        <v>57</v>
+      <c r="B18" s="40" t="s">
+        <v>67</v>
       </c>
       <c r="C18" s="11"/>
       <c r="D18" s="11"/>
       <c r="E18" s="12"/>
     </row>
     <row r="19">
-      <c r="A19" s="39"/>
-      <c r="B19" s="39"/>
-      <c r="C19" s="39"/>
-      <c r="D19" s="39"/>
-      <c r="E19" s="39"/>
+      <c r="A19" s="41"/>
+      <c r="B19" s="41"/>
+      <c r="C19" s="41"/>
+      <c r="D19" s="41"/>
+      <c r="E19" s="41"/>
     </row>
     <row r="21" ht="15.75" customHeight="1"/>
     <row r="22" ht="15.75" customHeight="1"/>
@@ -31229,8 +31362,8 @@
       <c r="Z1" s="1"/>
     </row>
     <row r="2" ht="24.0" customHeight="1">
-      <c r="A2" s="40" t="s">
-        <v>58</v>
+      <c r="A2" s="42" t="s">
+        <v>68</v>
       </c>
       <c r="B2" s="11"/>
       <c r="C2" s="11"/>
@@ -31238,25 +31371,25 @@
       <c r="E2" s="11"/>
       <c r="F2" s="11"/>
       <c r="G2" s="12"/>
-      <c r="H2" s="41"/>
-      <c r="I2" s="41"/>
-      <c r="J2" s="41"/>
-      <c r="K2" s="41"/>
-      <c r="L2" s="41"/>
-      <c r="M2" s="41"/>
-      <c r="N2" s="41"/>
-      <c r="O2" s="41"/>
-      <c r="P2" s="41"/>
-      <c r="Q2" s="41"/>
-      <c r="R2" s="41"/>
-      <c r="S2" s="41"/>
-      <c r="T2" s="41"/>
-      <c r="U2" s="41"/>
-      <c r="V2" s="41"/>
-      <c r="W2" s="41"/>
-      <c r="X2" s="41"/>
-      <c r="Y2" s="41"/>
-      <c r="Z2" s="41"/>
+      <c r="H2" s="43"/>
+      <c r="I2" s="43"/>
+      <c r="J2" s="43"/>
+      <c r="K2" s="43"/>
+      <c r="L2" s="43"/>
+      <c r="M2" s="43"/>
+      <c r="N2" s="43"/>
+      <c r="O2" s="43"/>
+      <c r="P2" s="43"/>
+      <c r="Q2" s="43"/>
+      <c r="R2" s="43"/>
+      <c r="S2" s="43"/>
+      <c r="T2" s="43"/>
+      <c r="U2" s="43"/>
+      <c r="V2" s="43"/>
+      <c r="W2" s="43"/>
+      <c r="X2" s="43"/>
+      <c r="Y2" s="43"/>
+      <c r="Z2" s="43"/>
     </row>
     <row r="3" ht="24.0" customHeight="1">
       <c r="A3" s="1"/>
@@ -31287,19 +31420,19 @@
       <c r="Z3" s="1"/>
     </row>
     <row r="4" ht="24.0" customHeight="1">
-      <c r="A4" s="42" t="s">
-        <v>59</v>
+      <c r="A4" s="44" t="s">
+        <v>69</v>
       </c>
-      <c r="B4" s="43" t="s">
-        <v>60</v>
+      <c r="B4" s="45" t="s">
+        <v>70</v>
       </c>
       <c r="C4" s="11"/>
       <c r="D4" s="11"/>
-      <c r="E4" s="42" t="s">
-        <v>61</v>
+      <c r="E4" s="44" t="s">
+        <v>71</v>
       </c>
-      <c r="F4" s="22" t="s">
-        <v>28</v>
+      <c r="F4" s="23" t="s">
+        <v>35</v>
       </c>
       <c r="G4" s="12"/>
       <c r="H4" s="1"/>
@@ -31323,19 +31456,19 @@
       <c r="Z4" s="1"/>
     </row>
     <row r="5" ht="24.0" customHeight="1">
-      <c r="A5" s="42" t="s">
-        <v>62</v>
+      <c r="A5" s="44" t="s">
+        <v>72</v>
       </c>
-      <c r="B5" s="43" t="s">
-        <v>63</v>
+      <c r="B5" s="45" t="s">
+        <v>73</v>
       </c>
       <c r="C5" s="11"/>
       <c r="D5" s="11"/>
-      <c r="E5" s="42" t="s">
-        <v>64</v>
+      <c r="E5" s="44" t="s">
+        <v>74</v>
       </c>
-      <c r="F5" s="44" t="s">
-        <v>65</v>
+      <c r="F5" s="46" t="s">
+        <v>75</v>
       </c>
       <c r="G5" s="12"/>
       <c r="H5" s="1"/>
@@ -31359,10 +31492,10 @@
       <c r="Z5" s="1"/>
     </row>
     <row r="6" ht="24.0" customHeight="1">
-      <c r="A6" s="45" t="s">
-        <v>66</v>
+      <c r="A6" s="47" t="s">
+        <v>76</v>
       </c>
-      <c r="B6" s="46"/>
+      <c r="B6" s="48"/>
       <c r="C6" s="11"/>
       <c r="D6" s="11"/>
       <c r="E6" s="11"/>
@@ -31417,95 +31550,99 @@
       <c r="Z7" s="1"/>
     </row>
     <row r="8" ht="24.0" customHeight="1">
-      <c r="A8" s="47" t="s">
+      <c r="A8" s="49" t="s">
         <v>1</v>
       </c>
-      <c r="B8" s="47" t="s">
-        <v>67</v>
+      <c r="B8" s="49" t="s">
+        <v>77</v>
       </c>
-      <c r="C8" s="48" t="s">
-        <v>44</v>
+      <c r="C8" s="50" t="s">
+        <v>51</v>
       </c>
       <c r="D8" s="12"/>
-      <c r="E8" s="47" t="s">
-        <v>68</v>
+      <c r="E8" s="49" t="s">
+        <v>78</v>
       </c>
-      <c r="F8" s="47" t="s">
-        <v>69</v>
+      <c r="F8" s="49" t="s">
+        <v>79</v>
       </c>
       <c r="G8" s="3" t="s">
-        <v>70</v>
+        <v>80</v>
       </c>
-      <c r="H8" s="49"/>
-      <c r="I8" s="49"/>
-      <c r="J8" s="49"/>
-      <c r="K8" s="49"/>
-      <c r="L8" s="49"/>
-      <c r="M8" s="49"/>
-      <c r="N8" s="49"/>
-      <c r="O8" s="49"/>
-      <c r="P8" s="49"/>
-      <c r="Q8" s="49"/>
-      <c r="R8" s="49"/>
-      <c r="S8" s="49"/>
-      <c r="T8" s="49"/>
-      <c r="U8" s="49"/>
-      <c r="V8" s="49"/>
-      <c r="W8" s="49"/>
-      <c r="X8" s="49"/>
-      <c r="Y8" s="49"/>
-      <c r="Z8" s="49"/>
+      <c r="H8" s="51"/>
+      <c r="I8" s="51"/>
+      <c r="J8" s="51"/>
+      <c r="K8" s="51"/>
+      <c r="L8" s="51"/>
+      <c r="M8" s="51"/>
+      <c r="N8" s="51"/>
+      <c r="O8" s="51"/>
+      <c r="P8" s="51"/>
+      <c r="Q8" s="51"/>
+      <c r="R8" s="51"/>
+      <c r="S8" s="51"/>
+      <c r="T8" s="51"/>
+      <c r="U8" s="51"/>
+      <c r="V8" s="51"/>
+      <c r="W8" s="51"/>
+      <c r="X8" s="51"/>
+      <c r="Y8" s="51"/>
+      <c r="Z8" s="51"/>
     </row>
     <row r="9" ht="24.0" customHeight="1">
-      <c r="A9" s="36"/>
-      <c r="B9" s="36"/>
-      <c r="C9" s="50" t="s">
-        <v>71</v>
+      <c r="A9" s="38"/>
+      <c r="B9" s="38"/>
+      <c r="C9" s="52" t="s">
+        <v>81</v>
       </c>
-      <c r="D9" s="50" t="s">
-        <v>72</v>
+      <c r="D9" s="52" t="s">
+        <v>82</v>
       </c>
-      <c r="E9" s="36"/>
-      <c r="F9" s="36"/>
-      <c r="G9" s="51"/>
-      <c r="H9" s="49"/>
-      <c r="I9" s="49"/>
-      <c r="J9" s="49"/>
-      <c r="K9" s="49"/>
-      <c r="L9" s="49"/>
-      <c r="M9" s="49"/>
-      <c r="N9" s="49"/>
-      <c r="O9" s="49"/>
-      <c r="P9" s="49"/>
-      <c r="Q9" s="49"/>
-      <c r="R9" s="49"/>
-      <c r="S9" s="49"/>
-      <c r="T9" s="49"/>
-      <c r="U9" s="49"/>
-      <c r="V9" s="49"/>
-      <c r="W9" s="49"/>
-      <c r="X9" s="49"/>
-      <c r="Y9" s="49"/>
-      <c r="Z9" s="49"/>
+      <c r="E9" s="38"/>
+      <c r="F9" s="38"/>
+      <c r="G9" s="53"/>
+      <c r="H9" s="51"/>
+      <c r="I9" s="51"/>
+      <c r="J9" s="51"/>
+      <c r="K9" s="51"/>
+      <c r="L9" s="51"/>
+      <c r="M9" s="51"/>
+      <c r="N9" s="51"/>
+      <c r="O9" s="51"/>
+      <c r="P9" s="51"/>
+      <c r="Q9" s="51"/>
+      <c r="R9" s="51"/>
+      <c r="S9" s="51"/>
+      <c r="T9" s="51"/>
+      <c r="U9" s="51"/>
+      <c r="V9" s="51"/>
+      <c r="W9" s="51"/>
+      <c r="X9" s="51"/>
+      <c r="Y9" s="51"/>
+      <c r="Z9" s="51"/>
     </row>
     <row r="10" ht="24.0" customHeight="1">
-      <c r="A10" s="52" t="s">
+      <c r="A10" s="54" t="s">
         <v>10</v>
       </c>
       <c r="B10" s="9" t="s">
-        <v>73</v>
+        <v>83</v>
       </c>
       <c r="C10" s="9" t="s">
-        <v>74</v>
+        <v>84</v>
       </c>
       <c r="D10" s="9">
         <v>3.0</v>
       </c>
       <c r="E10" s="13" t="s">
-        <v>53</v>
+        <v>60</v>
       </c>
-      <c r="F10" s="9"/>
-      <c r="G10" s="9"/>
+      <c r="F10" s="13" t="s">
+        <v>61</v>
+      </c>
+      <c r="G10" s="13" t="s">
+        <v>4</v>
+      </c>
       <c r="H10" s="1"/>
       <c r="I10" s="1"/>
       <c r="J10" s="1"/>
@@ -31527,21 +31664,25 @@
       <c r="Z10" s="1"/>
     </row>
     <row r="11" ht="24.0" customHeight="1">
-      <c r="A11" s="35"/>
+      <c r="A11" s="36"/>
       <c r="B11" s="9" t="s">
-        <v>75</v>
+        <v>25</v>
       </c>
       <c r="C11" s="9" t="s">
-        <v>76</v>
+        <v>85</v>
       </c>
       <c r="D11" s="9">
         <v>3.0</v>
       </c>
       <c r="E11" s="13" t="s">
-        <v>53</v>
+        <v>60</v>
       </c>
-      <c r="F11" s="9"/>
-      <c r="G11" s="9"/>
+      <c r="F11" s="13" t="s">
+        <v>86</v>
+      </c>
+      <c r="G11" s="13" t="s">
+        <v>5</v>
+      </c>
       <c r="H11" s="1"/>
       <c r="I11" s="1"/>
       <c r="J11" s="1"/>
@@ -31563,21 +31704,25 @@
       <c r="Z11" s="1"/>
     </row>
     <row r="12" ht="24.0" customHeight="1">
-      <c r="A12" s="35"/>
+      <c r="A12" s="36"/>
       <c r="B12" s="9" t="s">
-        <v>77</v>
+        <v>30</v>
       </c>
       <c r="C12" s="13" t="s">
-        <v>78</v>
+        <v>87</v>
       </c>
       <c r="D12" s="13">
         <v>3.0</v>
       </c>
       <c r="E12" s="13" t="s">
-        <v>79</v>
+        <v>88</v>
       </c>
-      <c r="F12" s="9"/>
-      <c r="G12" s="9"/>
+      <c r="F12" s="13" t="s">
+        <v>86</v>
+      </c>
+      <c r="G12" s="13" t="s">
+        <v>5</v>
+      </c>
       <c r="H12" s="1"/>
       <c r="I12" s="1"/>
       <c r="J12" s="1"/>
@@ -31599,21 +31744,25 @@
       <c r="Z12" s="1"/>
     </row>
     <row r="13" ht="24.0" customHeight="1">
-      <c r="A13" s="36"/>
+      <c r="A13" s="38"/>
       <c r="B13" s="9" t="s">
-        <v>80</v>
+        <v>31</v>
       </c>
       <c r="C13" s="13" t="s">
-        <v>81</v>
+        <v>89</v>
       </c>
       <c r="D13" s="13">
-        <v>2.0</v>
+        <v>3.0</v>
       </c>
       <c r="E13" s="13" t="s">
-        <v>82</v>
+        <v>90</v>
       </c>
-      <c r="F13" s="9"/>
-      <c r="G13" s="9"/>
+      <c r="F13" s="13" t="s">
+        <v>86</v>
+      </c>
+      <c r="G13" s="13" t="s">
+        <v>5</v>
+      </c>
       <c r="H13" s="1"/>
       <c r="I13" s="1"/>
       <c r="J13" s="1"/>

</xml_diff>